<commit_message>
Polish Goldratt demo dashboard
</commit_message>
<xml_diff>
--- a/public/templates/goldratt-bottleneck-template.xlsx
+++ b/public/templates/goldratt-bottleneck-template.xlsx
@@ -9,7 +9,8 @@
     <sheet name="Динамика по периодам" sheetId="4" r:id="rId4"/>
     <sheet name="Загрузка команды" sheetId="5" r:id="rId5"/>
     <sheet name="Что уже пробовали" sheetId="6" r:id="rId6"/>
-    <sheet name="Пример заполнения" sheetId="7" r:id="rId7"/>
+    <sheet name="Экономика потерь" sheetId="7" r:id="rId7"/>
+    <sheet name="Пример заполнения" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -403,14 +404,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A18"/>
   <cols>
     <col min="1" max="1" width="80.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Инструкция по заполнению шаблона bottleneck / Теория ограничений</v>
+        <v>Инструкция по заполнению шаблона ограничения / Теория ограничений</v>
       </c>
     </row>
     <row r="2">
@@ -420,67 +421,87 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Что сюда вносить</v>
+        <v>Этот шаблон нужен, чтобы найти главное ограничение системы: этап, который ограничивает скорость всего процесса.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>1. Карта процесса: основные этапы потока от входа до результата.</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Метрики потока: время ожидания, очередь, загрузка, SLA.</v>
+        <v>Какие данные нужны</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. Динамика по периодам: лиды, обработка, продажи, выручка, потери.</v>
+        <v>1. Карта процесса: этапы от входа до результата.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>4. Загрузка команды: роли, норма, факт, риск перегрузки.</v>
+        <v>2. Метрики потока: вход/выход, ожидание, норма, очередь, загрузка команды.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>5. Что уже пробовали: какие меры запускали и что не сработало.</v>
+        <v>3. Динамика по периодам: лиды, обработка, диагностики/продажи, оплаты, выручка, потери.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>4. Загрузка команды: роли, норма, факт, риск перегрузки.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Как использовать</v>
+        <v>5. Что уже пробовали: меры, которые уже запускались.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>— Не удаляйте строки с этапами, если данных нет: оставьте их пустыми.</v>
+        <v>6. Экономика потерь: где теряется поток и во сколько это обходится.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>— Не объединяйте ячейки.</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>— Заполняйте фактические значения за один и тот же период.</v>
+        <v>Как использовать</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>— Не удаляйте строки с этапами, если данных нет: оставьте их пустыми.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>— Не объединяйте ячейки.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>— Заполняйте фактические значения за один и тот же период.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>— Если ограничение ещё неочевидно, всё равно загрузите карту потока и метрики: система найдёт очередь и перегрузку.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>— Важно: здесь нужна операционная диагностика потока, а не только финансовый итог.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1211,6 +1232,93 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Причина потерь</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Объём</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Потенциальная выручка</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Комментарий</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Лиды без контакта за SLA</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Потери без повторного касания</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Отложенные внедрения</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Потери на этапе КП / предложения</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H16"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>

</xml_diff>